<commit_message>
continued crop stage assessments
</commit_message>
<xml_diff>
--- a/management_data_collated.xlsx
+++ b/management_data_collated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizabethforbes/Documents/Hudson Carbon/eddy covariance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDD3594-899B-E544-BD40-AF526E411A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F349AB-C37E-2248-A88C-66F1D0DC1F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1740" yWindow="760" windowWidth="16700" windowHeight="18880" xr2:uid="{15DBAF59-A2B3-3F43-91A8-FD158E0B7656}"/>
   </bookViews>
@@ -313,7 +313,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -349,31 +349,52 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{941080AA-DDDE-F14D-9EC1-8F3DC7D0F295}">
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" style="1"/>
@@ -716,3154 +737,3303 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="A2" s="8">
         <v>43028</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="6">
         <v>10</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="7">
         <v>2017</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="6">
         <f t="shared" ref="D2:D29" si="0">A2-DATE(YEAR(A2), 1, 0)</f>
         <v>293</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I2" t="s">
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="J2" s="6">
+        <v>1</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
+      <c r="A3" s="9">
         <v>43054</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>11</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="7">
         <v>2017</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="6">
         <f t="shared" si="0"/>
         <v>319</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="J3" s="6">
+        <v>1</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4" s="8">
         <v>43084</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="6">
         <v>12</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="7">
         <v>2017</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="6">
         <f t="shared" si="0"/>
         <v>349</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I4" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="J4" s="6">
+        <v>1</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="A5" s="8">
         <v>43222</v>
       </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5" s="6">
+        <v>5</v>
+      </c>
+      <c r="C5" s="7">
         <v>2018</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <f t="shared" si="0"/>
         <v>122</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I5" t="s">
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
+      <c r="A6" s="10">
         <v>43228</v>
       </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="B6" s="6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7">
         <v>2018</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <f t="shared" si="0"/>
         <v>128</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="J6" s="6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
+      <c r="A7" s="10">
         <v>43235</v>
       </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="B7" s="6">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7">
         <v>2018</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <f t="shared" si="0"/>
         <v>135</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I7" t="s">
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="J7" s="6">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="A8" s="8">
         <v>43240</v>
       </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1">
+      <c r="B8" s="6">
+        <v>5</v>
+      </c>
+      <c r="C8" s="7">
         <v>2018</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="6">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I8" t="s">
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J8">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
+      <c r="J8" s="6">
+        <v>1</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
+      <c r="A9" s="9">
         <v>43240</v>
       </c>
-      <c r="B9">
-        <v>5</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="B9" s="6">
+        <v>5</v>
+      </c>
+      <c r="C9" s="7">
         <v>2018</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="6">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="6">
         <v>10</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
+      <c r="A10" s="10">
         <v>43247</v>
       </c>
-      <c r="B10">
-        <v>5</v>
-      </c>
-      <c r="C10" s="1">
+      <c r="B10" s="6">
+        <v>5</v>
+      </c>
+      <c r="C10" s="7">
         <v>2018</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="6">
         <f t="shared" si="0"/>
         <v>147</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I10" t="s">
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="J10" s="6">
+        <v>1</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
+      <c r="A11" s="10">
         <v>43265</v>
       </c>
-      <c r="B11">
-        <v>6</v>
-      </c>
-      <c r="C11" s="1">
+      <c r="B11" s="6">
+        <v>6</v>
+      </c>
+      <c r="C11" s="7">
         <v>2018</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="6">
         <f t="shared" si="0"/>
         <v>165</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I11" t="s">
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="J11" s="6">
+        <v>1</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="A12" s="8">
         <v>43399</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="6">
         <v>10</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="7">
         <v>2018</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="6">
         <f t="shared" si="0"/>
         <v>299</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="J12" s="6">
+        <v>1</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
+      <c r="A13" s="9">
         <v>43400</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="6">
         <v>10</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="7">
         <v>2018</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="6">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13" t="s">
+      <c r="J13" s="6">
+        <v>1</v>
+      </c>
+      <c r="K13" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
+      <c r="A14" s="8">
         <v>43593</v>
       </c>
-      <c r="B14">
-        <v>5</v>
-      </c>
-      <c r="C14" s="1">
+      <c r="B14" s="6">
+        <v>5</v>
+      </c>
+      <c r="C14" s="7">
         <v>2019</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="6">
         <f t="shared" si="0"/>
         <v>128</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I14" t="s">
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14" t="s">
+      <c r="J14" s="6">
+        <v>1</v>
+      </c>
+      <c r="K14" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
+      <c r="A15" s="8">
         <v>43594</v>
       </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-      <c r="C15" s="1">
+      <c r="B15" s="6">
+        <v>5</v>
+      </c>
+      <c r="C15" s="7">
         <v>2019</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="6">
         <f t="shared" si="0"/>
         <v>129</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15" t="s">
+      <c r="J15" s="6">
+        <v>1</v>
+      </c>
+      <c r="K15" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="A16" s="8">
         <v>43594</v>
       </c>
-      <c r="B16">
-        <v>5</v>
-      </c>
-      <c r="C16" s="1">
+      <c r="B16" s="6">
+        <v>5</v>
+      </c>
+      <c r="C16" s="7">
         <v>2019</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="6">
         <f t="shared" si="0"/>
         <v>129</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I16" t="s">
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="J16">
-        <v>1</v>
-      </c>
-      <c r="K16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+      <c r="J16" s="6">
+        <v>1</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="8">
         <v>43775</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="6">
         <v>11</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="7">
         <v>2019</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="6">
         <f t="shared" si="0"/>
         <v>310</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J17">
-        <v>1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="2">
+      <c r="J17" s="6">
+        <v>1</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="8">
         <v>43780</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="6">
         <v>11</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="7">
         <v>2019</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="6">
         <f t="shared" si="0"/>
         <v>315</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J18">
-        <v>1</v>
-      </c>
-      <c r="K18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
+      <c r="J18" s="6">
+        <v>1</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="8">
         <v>43917</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="6">
         <v>3</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="7">
         <v>2020</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="6">
         <f t="shared" si="0"/>
         <v>87</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I19" t="s">
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="J19">
-        <v>1</v>
-      </c>
-      <c r="K19" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="9">
+      <c r="J19" s="6">
+        <v>1</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="8">
         <v>43919</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="6">
         <v>3</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="7">
         <v>2020</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="6">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J20" s="10">
-        <v>1</v>
-      </c>
-      <c r="K20" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="9">
+      <c r="J20" s="6">
+        <v>1</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L20" s="4"/>
+    </row>
+    <row r="21" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="8">
         <v>43919</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="6">
         <v>3</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="7">
         <v>2019</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="6">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J21" s="10">
-        <v>1</v>
-      </c>
-      <c r="K21" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="9">
+      <c r="J21" s="6">
+        <v>1</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L21" s="4"/>
+    </row>
+    <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="8">
         <v>43938</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="6">
         <v>4</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="7">
         <v>2020</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="6">
         <f t="shared" si="0"/>
         <v>108</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="J22" s="10">
-        <v>1</v>
-      </c>
-      <c r="K22" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12">
+      <c r="J22" s="6">
+        <v>1</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L22" s="4"/>
+    </row>
+    <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="8">
         <v>44021</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="6">
         <v>7</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="7">
         <v>2020</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="6">
         <f t="shared" si="0"/>
         <v>191</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="H23" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I23" s="13" t="s">
+      <c r="I23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J23" s="13">
-        <v>1</v>
-      </c>
-      <c r="K23" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="9">
+      <c r="J23" s="6">
+        <v>1</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L23" s="5"/>
+    </row>
+    <row r="24" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="8">
         <v>44089</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="6">
         <v>9</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="7">
         <v>2020</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="6">
         <f t="shared" si="0"/>
         <v>259</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="J24" s="10">
-        <v>1</v>
-      </c>
-      <c r="K24" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="15">
+      <c r="J24" s="6">
+        <v>1</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L24" s="4"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" s="8">
         <v>44090</v>
       </c>
-      <c r="B25" s="16">
+      <c r="B25" s="6">
         <v>9</v>
       </c>
-      <c r="C25" s="17">
+      <c r="C25" s="7">
         <v>2020</v>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="6">
         <f t="shared" si="0"/>
         <v>260</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="F25" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="16" t="s">
+      <c r="H25" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I25" s="16" t="s">
+      <c r="I25" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="J25" s="16">
-        <v>1</v>
-      </c>
-      <c r="K25" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="15">
+      <c r="J25" s="6">
+        <v>1</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" s="8">
         <v>44352</v>
       </c>
-      <c r="B26" s="16">
-        <v>6</v>
-      </c>
-      <c r="C26" s="17">
+      <c r="B26" s="6">
+        <v>6</v>
+      </c>
+      <c r="C26" s="7">
         <v>2021</v>
       </c>
-      <c r="D26" s="16">
+      <c r="D26" s="6">
         <f t="shared" si="0"/>
         <v>156</v>
       </c>
-      <c r="E26" s="16" t="s">
+      <c r="E26" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="F26" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H26" s="16" t="s">
+      <c r="H26" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I26" s="16" t="s">
+      <c r="I26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J26" s="16">
-        <v>1</v>
-      </c>
-      <c r="K26" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="15">
+      <c r="J26" s="6">
+        <v>1</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" s="8">
         <v>44418</v>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="6">
         <v>8</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C27" s="7">
         <v>2021</v>
       </c>
-      <c r="D27" s="16">
+      <c r="D27" s="6">
         <f t="shared" si="0"/>
         <v>222</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="E27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F27" s="16" t="s">
+      <c r="F27" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H27" s="16" t="s">
+      <c r="H27" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I27" s="16" t="s">
+      <c r="I27" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J27" s="16">
-        <v>1</v>
-      </c>
-      <c r="K27" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
+      <c r="J27" s="6">
+        <v>1</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" s="8">
         <v>43179</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="6">
         <v>3</v>
       </c>
-      <c r="C28" s="1">
+      <c r="C28" s="7">
         <v>2018</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="6">
         <f t="shared" si="0"/>
         <v>79</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I28" t="s">
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="J28">
-        <v>1</v>
-      </c>
-      <c r="K28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29" s="2">
+      <c r="J28" s="6">
+        <v>1</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" s="8">
         <v>43220</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="6">
         <v>4</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="7">
         <v>2018</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="6">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I29" t="s">
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="J29">
-        <v>1</v>
-      </c>
-      <c r="K29" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" s="2">
+      <c r="J29" s="6">
+        <v>1</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" s="8">
         <v>43221</v>
       </c>
-      <c r="B30">
-        <v>5</v>
-      </c>
-      <c r="C30" s="1">
+      <c r="B30" s="6">
+        <v>5</v>
+      </c>
+      <c r="C30" s="7">
         <v>2018</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="6">
         <f t="shared" ref="D30:D61" si="1">A30-DATE(YEAR(A30), 1, 0)</f>
         <v>121</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I30" t="s">
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J30">
-        <v>1</v>
-      </c>
-      <c r="K30" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="2">
+      <c r="J30" s="6">
+        <v>1</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" s="8">
         <v>43230</v>
       </c>
-      <c r="B31">
-        <v>5</v>
-      </c>
-      <c r="C31" s="1">
+      <c r="B31" s="6">
+        <v>5</v>
+      </c>
+      <c r="C31" s="7">
         <v>2018</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="6">
         <f t="shared" si="1"/>
         <v>130</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="J31">
-        <v>1</v>
-      </c>
-      <c r="K31" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="2">
+      <c r="J31" s="6">
+        <v>1</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32" s="8">
         <v>43232</v>
       </c>
-      <c r="B32">
-        <v>5</v>
-      </c>
-      <c r="C32" s="1">
+      <c r="B32" s="6">
+        <v>5</v>
+      </c>
+      <c r="C32" s="7">
         <v>2018</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="6">
         <f t="shared" si="1"/>
         <v>132</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I32" t="s">
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J32">
+      <c r="J32" s="6">
         <v>2</v>
       </c>
-      <c r="K32" t="s">
+      <c r="K32" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A33" s="2">
+      <c r="A33" s="8">
         <v>43278</v>
       </c>
-      <c r="B33">
-        <v>6</v>
-      </c>
-      <c r="C33" s="1">
+      <c r="B33" s="6">
+        <v>6</v>
+      </c>
+      <c r="C33" s="7">
         <v>2018</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="6">
         <f t="shared" si="1"/>
         <v>178</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I33" t="s">
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J33">
-        <v>1</v>
-      </c>
-      <c r="K33" t="s">
+      <c r="J33" s="6">
+        <v>1</v>
+      </c>
+      <c r="K33" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="2">
+      <c r="A34" s="8">
         <v>43279</v>
       </c>
-      <c r="B34">
-        <v>6</v>
-      </c>
-      <c r="C34" s="1">
+      <c r="B34" s="6">
+        <v>6</v>
+      </c>
+      <c r="C34" s="7">
         <v>2018</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="6">
         <f t="shared" si="1"/>
         <v>179</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I34" t="s">
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="J34">
-        <v>1</v>
-      </c>
-      <c r="K34" t="s">
+      <c r="J34" s="6">
+        <v>1</v>
+      </c>
+      <c r="K34" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
+      <c r="A35" s="8">
         <v>43377</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="6">
         <v>10</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="7">
         <v>2018</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="6">
         <f t="shared" si="1"/>
         <v>277</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="J35">
-        <v>1</v>
-      </c>
-      <c r="K35" t="s">
+      <c r="J35" s="6">
+        <v>1</v>
+      </c>
+      <c r="K35" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
+      <c r="A36" s="8">
         <v>43556</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="6">
         <v>4</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" s="7">
         <v>2019</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="6">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I36" t="s">
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J36">
-        <v>1</v>
-      </c>
-      <c r="K36" t="s">
+      <c r="J36" s="6">
+        <v>1</v>
+      </c>
+      <c r="K36" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
+      <c r="A37" s="8">
         <v>43559</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="6">
         <v>4</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" s="7">
         <v>2019</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="6">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I37" t="s">
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="J37">
-        <v>1</v>
-      </c>
-      <c r="K37" t="s">
+      <c r="J37" s="6">
+        <v>1</v>
+      </c>
+      <c r="K37" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
+      <c r="A38" s="8">
         <v>43617</v>
       </c>
-      <c r="B38">
-        <v>6</v>
-      </c>
-      <c r="C38" s="1">
+      <c r="B38" s="6">
+        <v>6</v>
+      </c>
+      <c r="C38" s="7">
         <v>2019</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="6">
         <f t="shared" si="1"/>
         <v>152</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H38" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I38" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J38">
-        <v>1</v>
-      </c>
-      <c r="K38" t="s">
+      <c r="J38" s="6">
+        <v>1</v>
+      </c>
+      <c r="K38" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
+      <c r="A39" s="8">
         <v>43739</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="6">
         <v>10</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="7">
         <v>2019</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="6">
         <f t="shared" si="1"/>
         <v>274</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H39" t="s">
+      <c r="H39" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J39">
-        <v>1</v>
-      </c>
-      <c r="K39" t="s">
+      <c r="J39" s="6">
+        <v>1</v>
+      </c>
+      <c r="K39" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
+      <c r="A40" s="8">
         <v>43753</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="6">
         <v>10</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" s="7">
         <v>2019</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="6">
         <f t="shared" si="1"/>
         <v>288</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H40" t="s">
+      <c r="H40" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="J40">
-        <v>1</v>
-      </c>
-      <c r="K40" t="s">
+      <c r="J40" s="6">
+        <v>1</v>
+      </c>
+      <c r="K40" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
+      <c r="A41" s="8">
         <v>43922</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="6">
         <v>4</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" s="7">
         <v>2020</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="6">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G41" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H41" t="s">
+      <c r="H41" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I41" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J41">
-        <v>1</v>
-      </c>
-      <c r="K41" t="s">
+      <c r="J41" s="6">
+        <v>1</v>
+      </c>
+      <c r="K41" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
+      <c r="A42" s="8">
         <v>43922</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="6">
         <v>4</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42" s="7">
         <v>2020</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="6">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I42" t="s">
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J42">
-        <v>1</v>
-      </c>
-      <c r="K42" t="s">
+      <c r="J42" s="6">
+        <v>1</v>
+      </c>
+      <c r="K42" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A43" s="2">
+      <c r="A43" s="8">
         <v>44013</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="6">
         <v>7</v>
       </c>
-      <c r="C43" s="1">
+      <c r="C43" s="7">
         <v>2020</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="6">
         <f t="shared" si="1"/>
         <v>183</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H43" t="s">
+      <c r="H43" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I43" t="s">
+      <c r="I43" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J43">
-        <v>1</v>
-      </c>
-      <c r="K43" t="s">
+      <c r="J43" s="6">
+        <v>1</v>
+      </c>
+      <c r="K43" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A44" s="2">
+      <c r="A44" s="8">
         <v>44027</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="6">
         <v>7</v>
       </c>
-      <c r="C44" s="1">
+      <c r="C44" s="7">
         <v>2020</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="6">
         <f t="shared" si="1"/>
         <v>197</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I44" t="s">
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J44">
-        <v>1</v>
-      </c>
-      <c r="K44" t="s">
+      <c r="J44" s="6">
+        <v>1</v>
+      </c>
+      <c r="K44" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A45" s="2">
+      <c r="A45" s="8">
         <v>44032</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="6">
         <v>7</v>
       </c>
-      <c r="C45" s="1">
+      <c r="C45" s="7">
         <v>2020</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="6">
         <f t="shared" si="1"/>
         <v>202</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G45" t="s">
+      <c r="G45" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H45" t="s">
+      <c r="H45" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="J45">
-        <v>1</v>
-      </c>
-      <c r="K45" t="s">
+      <c r="J45" s="6">
+        <v>1</v>
+      </c>
+      <c r="K45" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A46" s="2">
+      <c r="A46" s="8">
         <v>44287</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="6">
         <v>4</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" s="7">
         <v>2021</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="6">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I46" t="s">
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+      <c r="I46" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J46">
-        <v>1</v>
-      </c>
-      <c r="K46" t="s">
+      <c r="J46" s="6">
+        <v>1</v>
+      </c>
+      <c r="K46" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A47" s="2">
+      <c r="A47" s="8">
         <v>44348</v>
       </c>
-      <c r="B47">
-        <v>6</v>
-      </c>
-      <c r="C47" s="1">
+      <c r="B47" s="6">
+        <v>6</v>
+      </c>
+      <c r="C47" s="7">
         <v>2021</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="6">
         <f t="shared" si="1"/>
         <v>152</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G47" t="s">
+      <c r="G47" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H47" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I47" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J47">
-        <v>1</v>
-      </c>
-      <c r="K47" t="s">
+      <c r="J47" s="6">
+        <v>1</v>
+      </c>
+      <c r="K47" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
+      <c r="A48" s="8">
         <v>44470</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="6">
         <v>10</v>
       </c>
-      <c r="C48" s="1">
+      <c r="C48" s="7">
         <v>2021</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="6">
         <f t="shared" si="1"/>
         <v>274</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G48" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H48" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J48">
-        <v>1</v>
-      </c>
-      <c r="K48" t="s">
+      <c r="J48" s="6">
+        <v>1</v>
+      </c>
+      <c r="K48" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" s="5">
+      <c r="A49" s="11">
         <v>43237</v>
       </c>
-      <c r="B49">
-        <v>5</v>
-      </c>
-      <c r="C49" s="1">
+      <c r="B49" s="6">
+        <v>5</v>
+      </c>
+      <c r="C49" s="7">
         <v>2018</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="6">
         <f t="shared" si="1"/>
         <v>137</v>
       </c>
-      <c r="E49" t="s">
-        <v>6</v>
-      </c>
-      <c r="F49" t="s">
-        <v>5</v>
-      </c>
-      <c r="I49" t="s">
-        <v>5</v>
-      </c>
-      <c r="J49">
+      <c r="E49" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J49" s="6">
         <v>21</v>
       </c>
-      <c r="K49" t="s">
+      <c r="K49" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" s="5">
+      <c r="A50" s="11">
         <v>43258</v>
       </c>
-      <c r="B50">
-        <v>6</v>
-      </c>
-      <c r="C50" s="1">
+      <c r="B50" s="6">
+        <v>6</v>
+      </c>
+      <c r="C50" s="7">
         <v>2018</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="6">
         <f t="shared" si="1"/>
         <v>158</v>
       </c>
-      <c r="E50" t="s">
-        <v>6</v>
-      </c>
-      <c r="F50" t="s">
-        <v>5</v>
-      </c>
-      <c r="I50" t="s">
-        <v>5</v>
-      </c>
-      <c r="J50">
+      <c r="E50" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J50" s="6">
         <v>20</v>
       </c>
-      <c r="K50" t="s">
+      <c r="K50" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A51" s="5">
+      <c r="A51" s="11">
         <v>43261</v>
       </c>
-      <c r="B51">
-        <v>6</v>
-      </c>
-      <c r="C51" s="1">
+      <c r="B51" s="6">
+        <v>6</v>
+      </c>
+      <c r="C51" s="7">
         <v>2018</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="6">
         <f t="shared" si="1"/>
         <v>161</v>
       </c>
-      <c r="E51" t="s">
-        <v>6</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="E51" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I51" t="s">
+      <c r="G51" s="6"/>
+      <c r="H51" s="6"/>
+      <c r="I51" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J51">
-        <v>1</v>
-      </c>
-      <c r="K51" t="s">
+      <c r="J51" s="6">
+        <v>1</v>
+      </c>
+      <c r="K51" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A52" s="5">
+      <c r="A52" s="11">
         <v>43262</v>
       </c>
-      <c r="B52">
-        <v>6</v>
-      </c>
-      <c r="C52" s="1">
+      <c r="B52" s="6">
+        <v>6</v>
+      </c>
+      <c r="C52" s="7">
         <v>2018</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="6">
         <f t="shared" si="1"/>
         <v>162</v>
       </c>
-      <c r="E52" t="s">
-        <v>6</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="E52" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F52" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I52" t="s">
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J52">
-        <v>1</v>
-      </c>
-      <c r="K52" t="s">
+      <c r="J52" s="6">
+        <v>1</v>
+      </c>
+      <c r="K52" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" s="5">
+      <c r="A53" s="11">
         <v>43265</v>
       </c>
-      <c r="B53">
-        <v>6</v>
-      </c>
-      <c r="C53" s="1">
+      <c r="B53" s="6">
+        <v>6</v>
+      </c>
+      <c r="C53" s="7">
         <v>2018</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="6">
         <f t="shared" si="1"/>
         <v>165</v>
       </c>
-      <c r="E53" t="s">
-        <v>6</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="E53" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I53" t="s">
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J53">
-        <v>1</v>
-      </c>
-      <c r="K53" t="s">
+      <c r="J53" s="6">
+        <v>1</v>
+      </c>
+      <c r="K53" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A54" s="5">
+      <c r="A54" s="11">
         <v>43269</v>
       </c>
-      <c r="B54">
-        <v>6</v>
-      </c>
-      <c r="C54" s="1">
+      <c r="B54" s="6">
+        <v>6</v>
+      </c>
+      <c r="C54" s="7">
         <v>2018</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="6">
         <f t="shared" si="1"/>
         <v>169</v>
       </c>
-      <c r="E54" t="s">
-        <v>6</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="E54" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F54" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I54" t="s">
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J54">
+      <c r="J54" s="6">
         <v>2</v>
       </c>
-      <c r="K54" t="s">
+      <c r="K54" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A55" s="5">
+      <c r="A55" s="11">
         <v>43333</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="6">
         <v>8</v>
       </c>
-      <c r="C55" s="1">
+      <c r="C55" s="7">
         <v>2018</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="6">
         <f t="shared" si="1"/>
         <v>233</v>
       </c>
-      <c r="E55" t="s">
-        <v>6</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="E55" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F55" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I55" t="s">
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J55">
-        <v>1</v>
-      </c>
-      <c r="K55" t="s">
+      <c r="J55" s="6">
+        <v>1</v>
+      </c>
+      <c r="K55" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A56" s="5">
+      <c r="A56" s="11">
         <v>43336</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="6">
         <v>8</v>
       </c>
-      <c r="C56" s="1">
+      <c r="C56" s="7">
         <v>2018</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="6">
         <f t="shared" si="1"/>
         <v>236</v>
       </c>
-      <c r="E56" t="s">
-        <v>6</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="E56" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I56" t="s">
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J56">
-        <v>1</v>
-      </c>
-      <c r="K56" t="s">
+      <c r="J56" s="6">
+        <v>1</v>
+      </c>
+      <c r="K56" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A57" s="5">
+      <c r="A57" s="11">
         <v>43340</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="6">
         <v>8</v>
       </c>
-      <c r="C57" s="1">
+      <c r="C57" s="7">
         <v>2018</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="6">
         <f t="shared" si="1"/>
         <v>240</v>
       </c>
-      <c r="E57" t="s">
-        <v>6</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="E57" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I57" t="s">
+      <c r="G57" s="6"/>
+      <c r="H57" s="6"/>
+      <c r="I57" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J57">
-        <v>1</v>
-      </c>
-      <c r="K57" t="s">
+      <c r="J57" s="6">
+        <v>1</v>
+      </c>
+      <c r="K57" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A58" s="5">
+      <c r="A58" s="11">
         <v>43397</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="6">
         <v>10</v>
       </c>
-      <c r="C58" s="1">
+      <c r="C58" s="7">
         <v>2018</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="6">
         <f t="shared" si="1"/>
         <v>297</v>
       </c>
-      <c r="E58" t="s">
-        <v>6</v>
-      </c>
-      <c r="F58" t="s">
-        <v>5</v>
-      </c>
-      <c r="I58" t="s">
-        <v>5</v>
-      </c>
-      <c r="J58" t="s">
-        <v>57</v>
-      </c>
-      <c r="K58" t="s">
+      <c r="E58" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J58" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K58" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A59" s="2">
+      <c r="A59" s="8">
         <v>43586</v>
       </c>
-      <c r="B59">
-        <v>5</v>
-      </c>
-      <c r="C59" s="1">
+      <c r="B59" s="6">
+        <v>5</v>
+      </c>
+      <c r="C59" s="7">
         <v>2019</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="6">
         <f t="shared" si="1"/>
         <v>121</v>
       </c>
-      <c r="E59" t="s">
-        <v>6</v>
-      </c>
-      <c r="F59" t="s">
-        <v>5</v>
-      </c>
-      <c r="I59" t="s">
-        <v>5</v>
-      </c>
-      <c r="J59">
+      <c r="E59" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G59" s="6"/>
+      <c r="H59" s="6"/>
+      <c r="I59" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J59" s="6">
         <v>14</v>
       </c>
-      <c r="K59" t="s">
+      <c r="K59" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A60" s="2">
+      <c r="A60" s="8">
         <v>43600</v>
       </c>
-      <c r="B60">
-        <v>5</v>
-      </c>
-      <c r="C60" s="1">
+      <c r="B60" s="6">
+        <v>5</v>
+      </c>
+      <c r="C60" s="7">
         <v>2019</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="6">
         <f t="shared" si="1"/>
         <v>135</v>
       </c>
-      <c r="E60" t="s">
-        <v>6</v>
-      </c>
-      <c r="F60" t="s">
-        <v>5</v>
-      </c>
-      <c r="I60" t="s">
-        <v>5</v>
-      </c>
-      <c r="J60">
-        <v>5</v>
-      </c>
-      <c r="K60" t="s">
+      <c r="E60" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G60" s="6"/>
+      <c r="H60" s="6"/>
+      <c r="I60" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J60" s="6">
+        <v>5</v>
+      </c>
+      <c r="K60" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A61" s="2">
+      <c r="A61" s="8">
         <v>43605</v>
       </c>
-      <c r="B61">
-        <v>5</v>
-      </c>
-      <c r="C61" s="1">
+      <c r="B61" s="6">
+        <v>5</v>
+      </c>
+      <c r="C61" s="7">
         <v>2019</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="6">
         <f t="shared" si="1"/>
         <v>140</v>
       </c>
-      <c r="E61" t="s">
-        <v>6</v>
-      </c>
-      <c r="F61" t="s">
-        <v>5</v>
-      </c>
-      <c r="I61" t="s">
-        <v>5</v>
-      </c>
-      <c r="J61">
+      <c r="E61" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J61" s="6">
         <v>15</v>
       </c>
-      <c r="K61" t="s">
+      <c r="K61" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A62" s="2">
+      <c r="A62" s="8">
         <v>43616</v>
       </c>
-      <c r="B62">
-        <v>5</v>
-      </c>
-      <c r="C62" s="1">
+      <c r="B62" s="6">
+        <v>5</v>
+      </c>
+      <c r="C62" s="7">
         <v>2019</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="6">
         <f t="shared" ref="D62:D90" si="2">A62-DATE(YEAR(A62), 1, 0)</f>
         <v>151</v>
       </c>
-      <c r="E62" t="s">
-        <v>6</v>
-      </c>
-      <c r="F62" t="s">
+      <c r="E62" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F62" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I62" t="s">
+      <c r="G62" s="6"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J62">
-        <v>1</v>
-      </c>
-      <c r="K62" t="s">
+      <c r="J62" s="6">
+        <v>1</v>
+      </c>
+      <c r="K62" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A63" s="2">
+      <c r="A63" s="8">
         <v>43617</v>
       </c>
-      <c r="B63">
-        <v>6</v>
-      </c>
-      <c r="C63" s="1">
+      <c r="B63" s="6">
+        <v>6</v>
+      </c>
+      <c r="C63" s="7">
         <v>2019</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="6">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
-      <c r="E63" t="s">
-        <v>6</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="E63" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I63" t="s">
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J63">
-        <v>1</v>
-      </c>
-      <c r="K63" t="s">
+      <c r="J63" s="6">
+        <v>1</v>
+      </c>
+      <c r="K63" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A64" s="2">
+      <c r="A64" s="8">
         <v>43619</v>
       </c>
-      <c r="B64">
-        <v>6</v>
-      </c>
-      <c r="C64" s="1">
+      <c r="B64" s="6">
+        <v>6</v>
+      </c>
+      <c r="C64" s="7">
         <v>2019</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="6">
         <f t="shared" si="2"/>
         <v>154</v>
       </c>
-      <c r="E64" t="s">
-        <v>6</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="E64" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F64" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I64" t="s">
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J64">
-        <v>1</v>
-      </c>
-      <c r="K64" t="s">
+      <c r="J64" s="6">
+        <v>1</v>
+      </c>
+      <c r="K64" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A65" s="2">
+      <c r="A65" s="8">
         <v>43620</v>
       </c>
-      <c r="B65">
-        <v>6</v>
-      </c>
-      <c r="C65" s="1">
+      <c r="B65" s="6">
+        <v>6</v>
+      </c>
+      <c r="C65" s="7">
         <v>2019</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="6">
         <f t="shared" si="2"/>
         <v>155</v>
       </c>
-      <c r="E65" t="s">
-        <v>6</v>
-      </c>
-      <c r="F65" t="s">
+      <c r="E65" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I65" t="s">
+      <c r="G65" s="6"/>
+      <c r="H65" s="6"/>
+      <c r="I65" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J65">
-        <v>1</v>
-      </c>
-      <c r="K65" t="s">
+      <c r="J65" s="6">
+        <v>1</v>
+      </c>
+      <c r="K65" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A66" s="2">
+      <c r="A66" s="8">
         <v>43621</v>
       </c>
-      <c r="B66">
-        <v>6</v>
-      </c>
-      <c r="C66" s="1">
+      <c r="B66" s="6">
+        <v>6</v>
+      </c>
+      <c r="C66" s="7">
         <v>2019</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="6">
         <f t="shared" si="2"/>
         <v>156</v>
       </c>
-      <c r="E66" t="s">
-        <v>6</v>
-      </c>
-      <c r="F66" t="s">
-        <v>5</v>
-      </c>
-      <c r="I66" t="s">
-        <v>5</v>
-      </c>
-      <c r="J66">
-        <v>5</v>
-      </c>
-      <c r="K66" t="s">
+      <c r="E66" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G66" s="6"/>
+      <c r="H66" s="6"/>
+      <c r="I66" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J66" s="6">
+        <v>5</v>
+      </c>
+      <c r="K66" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A67" s="2">
+      <c r="A67" s="8">
         <v>43622</v>
       </c>
-      <c r="B67">
-        <v>6</v>
-      </c>
-      <c r="C67" s="1">
+      <c r="B67" s="6">
+        <v>6</v>
+      </c>
+      <c r="C67" s="7">
         <v>2019</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="6">
         <f t="shared" si="2"/>
         <v>157</v>
       </c>
-      <c r="E67" t="s">
-        <v>6</v>
-      </c>
-      <c r="F67" t="s">
+      <c r="E67" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I67" t="s">
+      <c r="G67" s="6"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J67">
-        <v>1</v>
-      </c>
-      <c r="K67" t="s">
+      <c r="J67" s="6">
+        <v>1</v>
+      </c>
+      <c r="K67" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A68" s="2">
+      <c r="A68" s="8">
         <v>43623</v>
       </c>
-      <c r="B68">
-        <v>6</v>
-      </c>
-      <c r="C68" s="1">
+      <c r="B68" s="6">
+        <v>6</v>
+      </c>
+      <c r="C68" s="7">
         <v>2019</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="6">
         <f t="shared" si="2"/>
         <v>158</v>
       </c>
-      <c r="E68" t="s">
-        <v>6</v>
-      </c>
-      <c r="F68" t="s">
+      <c r="E68" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F68" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I68" t="s">
+      <c r="G68" s="6"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J68">
-        <v>1</v>
-      </c>
-      <c r="K68" t="s">
+      <c r="J68" s="6">
+        <v>1</v>
+      </c>
+      <c r="K68" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A69" s="2">
+      <c r="A69" s="8">
         <v>43624</v>
       </c>
-      <c r="B69">
-        <v>6</v>
-      </c>
-      <c r="C69" s="1">
+      <c r="B69" s="6">
+        <v>6</v>
+      </c>
+      <c r="C69" s="7">
         <v>2019</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="6">
         <f t="shared" si="2"/>
         <v>159</v>
       </c>
-      <c r="E69" t="s">
-        <v>6</v>
-      </c>
-      <c r="F69" t="s">
-        <v>5</v>
-      </c>
-      <c r="I69" t="s">
-        <v>5</v>
-      </c>
-      <c r="J69">
+      <c r="E69" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G69" s="6"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J69" s="6">
         <v>12</v>
       </c>
-      <c r="K69" t="s">
+      <c r="K69" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A70" s="2">
+      <c r="A70" s="8">
         <v>43626</v>
       </c>
-      <c r="B70">
-        <v>6</v>
-      </c>
-      <c r="C70" s="1">
+      <c r="B70" s="6">
+        <v>6</v>
+      </c>
+      <c r="C70" s="7">
         <v>2019</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="6">
         <f t="shared" si="2"/>
         <v>161</v>
       </c>
-      <c r="E70" t="s">
-        <v>6</v>
-      </c>
-      <c r="F70" t="s">
-        <v>5</v>
-      </c>
-      <c r="I70" t="s">
-        <v>5</v>
-      </c>
-      <c r="J70">
+      <c r="E70" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J70" s="6">
         <v>13</v>
       </c>
-      <c r="K70" t="s">
+      <c r="K70" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A71" s="2">
+      <c r="A71" s="8">
         <v>43627</v>
       </c>
-      <c r="B71">
-        <v>6</v>
-      </c>
-      <c r="C71" s="1">
+      <c r="B71" s="6">
+        <v>6</v>
+      </c>
+      <c r="C71" s="7">
         <v>2019</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="6">
         <f t="shared" si="2"/>
         <v>162</v>
       </c>
-      <c r="E71" t="s">
-        <v>6</v>
-      </c>
-      <c r="F71" t="s">
+      <c r="E71" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I71" t="s">
+      <c r="G71" s="6"/>
+      <c r="H71" s="6"/>
+      <c r="I71" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J71">
-        <v>1</v>
-      </c>
-      <c r="K71" t="s">
+      <c r="J71" s="6">
+        <v>1</v>
+      </c>
+      <c r="K71" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A72" s="2">
+      <c r="A72" s="8">
         <v>43628</v>
       </c>
-      <c r="B72">
-        <v>6</v>
-      </c>
-      <c r="C72" s="1">
+      <c r="B72" s="6">
+        <v>6</v>
+      </c>
+      <c r="C72" s="7">
         <v>2019</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="6">
         <f t="shared" si="2"/>
         <v>163</v>
       </c>
-      <c r="E72" t="s">
-        <v>6</v>
-      </c>
-      <c r="F72" t="s">
+      <c r="E72" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F72" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I72" t="s">
+      <c r="G72" s="6"/>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J72">
-        <v>1</v>
-      </c>
-      <c r="K72" t="s">
+      <c r="J72" s="6">
+        <v>1</v>
+      </c>
+      <c r="K72" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A73" s="2">
+      <c r="A73" s="8">
         <v>43640</v>
       </c>
-      <c r="B73">
-        <v>6</v>
-      </c>
-      <c r="C73" s="1">
+      <c r="B73" s="6">
+        <v>6</v>
+      </c>
+      <c r="C73" s="7">
         <v>2019</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="6">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-      <c r="E73" t="s">
-        <v>6</v>
-      </c>
-      <c r="F73" t="s">
-        <v>5</v>
-      </c>
-      <c r="I73" t="s">
-        <v>5</v>
-      </c>
-      <c r="J73">
+      <c r="E73" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J73" s="6">
         <v>7</v>
       </c>
-      <c r="K73" t="s">
+      <c r="K73" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A74" s="2">
+      <c r="A74" s="8">
         <v>43647</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="6">
         <v>7</v>
       </c>
-      <c r="C74" s="1">
+      <c r="C74" s="7">
         <v>2019</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="6">
         <f t="shared" si="2"/>
         <v>182</v>
       </c>
-      <c r="E74" t="s">
-        <v>6</v>
-      </c>
-      <c r="F74" t="s">
-        <v>5</v>
-      </c>
-      <c r="I74" t="s">
-        <v>5</v>
-      </c>
-      <c r="J74">
+      <c r="E74" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G74" s="6"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J74" s="6">
         <v>15</v>
       </c>
-      <c r="K74" t="s">
+      <c r="K74" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A75" s="2">
+      <c r="A75" s="8">
         <v>43697</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="6">
         <v>8</v>
       </c>
-      <c r="C75" s="1">
+      <c r="C75" s="7">
         <v>2019</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="6">
         <f t="shared" si="2"/>
         <v>232</v>
       </c>
-      <c r="E75" t="s">
-        <v>6</v>
-      </c>
-      <c r="F75" t="s">
-        <v>5</v>
-      </c>
-      <c r="I75" t="s">
-        <v>5</v>
-      </c>
-      <c r="J75">
+      <c r="E75" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G75" s="6"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J75" s="6">
         <v>11</v>
       </c>
-      <c r="K75" t="s">
+      <c r="K75" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A76" s="2">
+      <c r="A76" s="8">
         <v>43708</v>
       </c>
-      <c r="B76">
+      <c r="B76" s="6">
         <v>8</v>
       </c>
-      <c r="C76" s="1">
+      <c r="C76" s="7">
         <v>2019</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="6">
         <f t="shared" si="2"/>
         <v>243</v>
       </c>
-      <c r="E76" t="s">
-        <v>6</v>
-      </c>
-      <c r="F76" t="s">
-        <v>5</v>
-      </c>
-      <c r="I76" t="s">
-        <v>5</v>
-      </c>
-      <c r="J76">
+      <c r="E76" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G76" s="6"/>
+      <c r="H76" s="6"/>
+      <c r="I76" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J76" s="6">
         <v>10</v>
       </c>
-      <c r="K76" t="s">
+      <c r="K76" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A77" s="2">
+      <c r="A77" s="8">
         <v>43714</v>
       </c>
-      <c r="B77">
+      <c r="B77" s="6">
         <v>9</v>
       </c>
-      <c r="C77" s="1">
+      <c r="C77" s="7">
         <v>2019</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="6">
         <f t="shared" si="2"/>
         <v>249</v>
       </c>
-      <c r="E77" t="s">
-        <v>6</v>
-      </c>
-      <c r="F77" t="s">
+      <c r="E77" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F77" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I77" t="s">
+      <c r="G77" s="6"/>
+      <c r="H77" s="6"/>
+      <c r="I77" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J77">
-        <v>1</v>
-      </c>
-      <c r="K77" t="s">
+      <c r="J77" s="6">
+        <v>1</v>
+      </c>
+      <c r="K77" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A78" s="2">
+      <c r="A78" s="8">
         <v>43717</v>
       </c>
-      <c r="B78">
+      <c r="B78" s="6">
         <v>9</v>
       </c>
-      <c r="C78" s="1">
+      <c r="C78" s="7">
         <v>2019</v>
       </c>
-      <c r="D78">
+      <c r="D78" s="6">
         <f t="shared" si="2"/>
         <v>252</v>
       </c>
-      <c r="E78" t="s">
-        <v>6</v>
-      </c>
-      <c r="F78" t="s">
+      <c r="E78" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F78" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I78" t="s">
+      <c r="G78" s="6"/>
+      <c r="H78" s="6"/>
+      <c r="I78" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J78">
-        <v>1</v>
-      </c>
-      <c r="K78" t="s">
+      <c r="J78" s="6">
+        <v>1</v>
+      </c>
+      <c r="K78" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A79" s="2">
+      <c r="A79" s="8">
         <v>43726</v>
       </c>
-      <c r="B79">
+      <c r="B79" s="6">
         <v>9</v>
       </c>
-      <c r="C79" s="1">
+      <c r="C79" s="7">
         <v>2019</v>
       </c>
-      <c r="D79">
+      <c r="D79" s="6">
         <f t="shared" si="2"/>
         <v>261</v>
       </c>
-      <c r="E79" t="s">
-        <v>6</v>
-      </c>
-      <c r="F79" t="s">
+      <c r="E79" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I79" t="s">
+      <c r="G79" s="6"/>
+      <c r="H79" s="6"/>
+      <c r="I79" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J79">
-        <v>1</v>
-      </c>
-      <c r="K79" t="s">
+      <c r="J79" s="6">
+        <v>1</v>
+      </c>
+      <c r="K79" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A80" s="2">
+      <c r="A80" s="8">
         <v>43727</v>
       </c>
-      <c r="B80">
+      <c r="B80" s="6">
         <v>9</v>
       </c>
-      <c r="C80" s="1">
+      <c r="C80" s="7">
         <v>2019</v>
       </c>
-      <c r="D80">
+      <c r="D80" s="6">
         <f t="shared" si="2"/>
         <v>262</v>
       </c>
-      <c r="E80" t="s">
-        <v>6</v>
-      </c>
-      <c r="F80" t="s">
+      <c r="E80" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F80" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I80" t="s">
+      <c r="G80" s="6"/>
+      <c r="H80" s="6"/>
+      <c r="I80" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J80">
-        <v>1</v>
-      </c>
-      <c r="K80" t="s">
+      <c r="J80" s="6">
+        <v>1</v>
+      </c>
+      <c r="K80" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A81" s="2">
+      <c r="A81" s="8">
         <v>43728</v>
       </c>
-      <c r="B81">
+      <c r="B81" s="6">
         <v>9</v>
       </c>
-      <c r="C81" s="1">
+      <c r="C81" s="7">
         <v>2019</v>
       </c>
-      <c r="D81">
+      <c r="D81" s="6">
         <f t="shared" si="2"/>
         <v>263</v>
       </c>
-      <c r="E81" t="s">
-        <v>6</v>
-      </c>
-      <c r="F81" t="s">
+      <c r="E81" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I81" t="s">
+      <c r="G81" s="6"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J81">
-        <v>1</v>
-      </c>
-      <c r="K81" t="s">
+      <c r="J81" s="6">
+        <v>1</v>
+      </c>
+      <c r="K81" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A82" s="2">
+      <c r="A82" s="8">
         <v>43756</v>
       </c>
-      <c r="B82">
+      <c r="B82" s="6">
         <v>10</v>
       </c>
-      <c r="C82" s="1">
+      <c r="C82" s="7">
         <v>2019</v>
       </c>
-      <c r="D82">
+      <c r="D82" s="6">
         <f t="shared" si="2"/>
         <v>291</v>
       </c>
-      <c r="E82" t="s">
-        <v>6</v>
-      </c>
-      <c r="F82" t="s">
-        <v>5</v>
-      </c>
-      <c r="I82" t="s">
-        <v>5</v>
-      </c>
-      <c r="J82">
+      <c r="E82" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G82" s="6"/>
+      <c r="H82" s="6"/>
+      <c r="I82" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J82" s="6">
         <v>18</v>
       </c>
-      <c r="K82" t="s">
+      <c r="K82" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A83" s="2">
+      <c r="A83" s="8">
         <v>43763</v>
       </c>
-      <c r="B83">
+      <c r="B83" s="6">
         <v>10</v>
       </c>
-      <c r="C83" s="1">
+      <c r="C83" s="7">
         <v>2019</v>
       </c>
-      <c r="D83">
+      <c r="D83" s="6">
         <f t="shared" si="2"/>
         <v>298</v>
       </c>
-      <c r="E83" t="s">
-        <v>6</v>
-      </c>
-      <c r="F83" t="s">
+      <c r="E83" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F83" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I83" t="s">
+      <c r="G83" s="6"/>
+      <c r="H83" s="6"/>
+      <c r="I83" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J83">
-        <v>1</v>
-      </c>
-      <c r="K83" t="s">
+      <c r="J83" s="6">
+        <v>1</v>
+      </c>
+      <c r="K83" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A84" s="2">
+      <c r="A84" s="8">
         <v>43772</v>
       </c>
-      <c r="B84">
+      <c r="B84" s="6">
         <v>11</v>
       </c>
-      <c r="C84" s="1">
+      <c r="C84" s="7">
         <v>2020</v>
       </c>
-      <c r="D84">
+      <c r="D84" s="6">
         <f t="shared" si="2"/>
         <v>307</v>
       </c>
-      <c r="E84" t="s">
-        <v>6</v>
-      </c>
-      <c r="F84" t="s">
+      <c r="E84" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F84" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I84" t="s">
+      <c r="G84" s="6"/>
+      <c r="H84" s="6"/>
+      <c r="I84" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J84">
-        <v>1</v>
-      </c>
-      <c r="K84" t="s">
+      <c r="J84" s="6">
+        <v>1</v>
+      </c>
+      <c r="K84" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A85" s="2">
+      <c r="A85" s="8">
         <v>43912</v>
       </c>
-      <c r="B85">
+      <c r="B85" s="6">
         <v>3</v>
       </c>
-      <c r="C85" s="1">
+      <c r="C85" s="7">
         <v>2020</v>
       </c>
-      <c r="D85">
+      <c r="D85" s="6">
         <f t="shared" si="2"/>
         <v>82</v>
       </c>
-      <c r="E85" t="s">
-        <v>6</v>
-      </c>
-      <c r="F85" t="s">
+      <c r="E85" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F85" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I85" t="s">
+      <c r="G85" s="6"/>
+      <c r="H85" s="6"/>
+      <c r="I85" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J85">
+      <c r="J85" s="6">
         <v>2</v>
       </c>
-      <c r="K85" t="s">
+      <c r="K85" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A86" s="2">
+      <c r="A86" s="8">
         <v>43929</v>
       </c>
-      <c r="B86">
+      <c r="B86" s="6">
         <v>4</v>
       </c>
-      <c r="C86" s="1">
+      <c r="C86" s="7">
         <v>2020</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="6">
         <f t="shared" si="2"/>
         <v>99</v>
       </c>
-      <c r="E86" t="s">
-        <v>6</v>
-      </c>
-      <c r="F86" t="s">
+      <c r="E86" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F86" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I86" t="s">
+      <c r="G86" s="6"/>
+      <c r="H86" s="6"/>
+      <c r="I86" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J86">
+      <c r="J86" s="6">
         <v>2</v>
       </c>
-      <c r="K86" t="s">
+      <c r="K86" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A87" s="2">
+      <c r="A87" s="8">
         <v>43971</v>
       </c>
-      <c r="B87">
-        <v>5</v>
-      </c>
-      <c r="C87" s="1">
+      <c r="B87" s="6">
+        <v>5</v>
+      </c>
+      <c r="C87" s="7">
         <v>2020</v>
       </c>
-      <c r="D87">
+      <c r="D87" s="6">
         <f t="shared" si="2"/>
         <v>141</v>
       </c>
-      <c r="E87" t="s">
-        <v>6</v>
-      </c>
-      <c r="F87" t="s">
+      <c r="E87" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F87" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I87" t="s">
+      <c r="G87" s="6"/>
+      <c r="H87" s="6"/>
+      <c r="I87" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J87">
-        <v>1</v>
-      </c>
-      <c r="K87" t="s">
+      <c r="J87" s="6">
+        <v>1</v>
+      </c>
+      <c r="K87" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A88" s="2">
+      <c r="A88" s="8">
         <v>43972</v>
       </c>
-      <c r="B88">
-        <v>5</v>
-      </c>
-      <c r="C88" s="1">
+      <c r="B88" s="6">
+        <v>5</v>
+      </c>
+      <c r="C88" s="7">
         <v>2020</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="6">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
-      <c r="E88" t="s">
-        <v>6</v>
-      </c>
-      <c r="F88" t="s">
+      <c r="E88" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F88" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I88" t="s">
+      <c r="G88" s="6"/>
+      <c r="H88" s="6"/>
+      <c r="I88" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J88">
-        <v>1</v>
-      </c>
-      <c r="K88" t="s">
+      <c r="J88" s="6">
+        <v>1</v>
+      </c>
+      <c r="K88" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A89" s="2">
+      <c r="A89" s="8">
         <v>43972</v>
       </c>
-      <c r="B89">
-        <v>5</v>
-      </c>
-      <c r="C89" s="1">
+      <c r="B89" s="6">
+        <v>5</v>
+      </c>
+      <c r="C89" s="7">
         <v>2020</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="6">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
-      <c r="E89" t="s">
-        <v>6</v>
-      </c>
-      <c r="F89" t="s">
+      <c r="E89" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F89" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I89" t="s">
+      <c r="G89" s="6"/>
+      <c r="H89" s="6"/>
+      <c r="I89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J89">
-        <v>1</v>
-      </c>
-      <c r="K89" t="s">
+      <c r="J89" s="6">
+        <v>1</v>
+      </c>
+      <c r="K89" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A90" s="2">
+      <c r="A90" s="8">
         <v>43973</v>
       </c>
-      <c r="B90">
-        <v>5</v>
-      </c>
-      <c r="C90" s="1">
+      <c r="B90" s="6">
+        <v>5</v>
+      </c>
+      <c r="C90" s="7">
         <v>2020</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="6">
         <f t="shared" si="2"/>
         <v>143</v>
       </c>
-      <c r="E90" t="s">
-        <v>6</v>
-      </c>
-      <c r="F90" t="s">
+      <c r="E90" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F90" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I90" t="s">
+      <c r="G90" s="6"/>
+      <c r="H90" s="6"/>
+      <c r="I90" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J90">
-        <v>1</v>
-      </c>
-      <c r="K90" t="s">
+      <c r="J90" s="6">
+        <v>1</v>
+      </c>
+      <c r="K90" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A91" s="6">
+      <c r="A91" s="12">
         <v>43975</v>
       </c>
-      <c r="B91" s="7">
-        <v>5</v>
-      </c>
-      <c r="C91" s="8">
+      <c r="B91" s="13">
+        <v>5</v>
+      </c>
+      <c r="C91" s="14">
         <v>2020</v>
       </c>
-      <c r="D91" s="7">
+      <c r="D91" s="13">
         <v>142</v>
       </c>
-      <c r="E91" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F91" s="7" t="s">
+      <c r="E91" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F91" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G91" s="7"/>
-      <c r="H91" s="7"/>
-      <c r="I91" s="7" t="s">
+      <c r="G91" s="13"/>
+      <c r="H91" s="13"/>
+      <c r="I91" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="J91" s="7">
-        <v>1</v>
-      </c>
-      <c r="K91" t="s">
+      <c r="J91" s="13">
+        <v>1</v>
+      </c>
+      <c r="K91" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A92" s="6">
+      <c r="A92" s="12">
         <v>43976</v>
       </c>
-      <c r="B92" s="7">
-        <v>5</v>
-      </c>
-      <c r="C92" s="8">
+      <c r="B92" s="13">
+        <v>5</v>
+      </c>
+      <c r="C92" s="14">
         <v>2020</v>
       </c>
-      <c r="D92" s="7">
+      <c r="D92" s="13">
         <v>142</v>
       </c>
-      <c r="E92" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F92" s="7" t="s">
+      <c r="E92" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F92" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G92" s="7"/>
-      <c r="H92" s="7"/>
-      <c r="I92" s="7" t="s">
+      <c r="G92" s="13"/>
+      <c r="H92" s="13"/>
+      <c r="I92" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="J92" s="7">
-        <v>1</v>
-      </c>
-      <c r="K92" t="s">
+      <c r="J92" s="13">
+        <v>1</v>
+      </c>
+      <c r="K92" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A93" s="2">
+      <c r="A93" s="8">
         <v>43977</v>
       </c>
-      <c r="B93">
-        <v>5</v>
-      </c>
-      <c r="C93" s="1">
+      <c r="B93" s="6">
+        <v>5</v>
+      </c>
+      <c r="C93" s="7">
         <v>2020</v>
       </c>
-      <c r="D93">
+      <c r="D93" s="6">
         <f>A93-DATE(YEAR(A93), 1, 0)</f>
         <v>147</v>
       </c>
-      <c r="E93" t="s">
-        <v>6</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="E93" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F93" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I93" t="s">
+      <c r="G93" s="6"/>
+      <c r="H93" s="6"/>
+      <c r="I93" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J93">
-        <v>1</v>
-      </c>
-      <c r="K93" t="s">
+      <c r="J93" s="6">
+        <v>1</v>
+      </c>
+      <c r="K93" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="2">
+      <c r="A94" s="8">
         <v>43977</v>
       </c>
-      <c r="B94">
-        <v>5</v>
-      </c>
-      <c r="C94" s="1">
+      <c r="B94" s="6">
+        <v>5</v>
+      </c>
+      <c r="C94" s="7">
         <v>2020</v>
       </c>
-      <c r="D94">
+      <c r="D94" s="6">
         <f>A94-DATE(YEAR(A94), 1, 0)</f>
         <v>147</v>
       </c>
-      <c r="E94" t="s">
-        <v>6</v>
-      </c>
-      <c r="F94" t="s">
+      <c r="E94" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F94" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I94" t="s">
+      <c r="G94" s="6"/>
+      <c r="H94" s="6"/>
+      <c r="I94" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="J94">
-        <v>1</v>
-      </c>
-      <c r="K94" t="s">
+      <c r="J94" s="6">
+        <v>1</v>
+      </c>
+      <c r="K94" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A95" s="6">
+      <c r="A95" s="12">
         <v>43978</v>
       </c>
-      <c r="B95" s="7">
-        <v>5</v>
-      </c>
-      <c r="C95" s="8">
+      <c r="B95" s="13">
+        <v>5</v>
+      </c>
+      <c r="C95" s="14">
         <v>2020</v>
       </c>
-      <c r="D95" s="7">
+      <c r="D95" s="13">
         <v>147</v>
       </c>
-      <c r="E95" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F95" s="7" t="s">
+      <c r="E95" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F95" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G95" s="7"/>
-      <c r="H95" s="7"/>
-      <c r="I95" s="7" t="s">
+      <c r="G95" s="13"/>
+      <c r="H95" s="13"/>
+      <c r="I95" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="J95" s="7">
-        <v>1</v>
-      </c>
-      <c r="K95" t="s">
+      <c r="J95" s="13">
+        <v>1</v>
+      </c>
+      <c r="K95" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A96" s="2">
+      <c r="A96" s="8">
         <v>43980</v>
       </c>
-      <c r="B96">
-        <v>5</v>
-      </c>
-      <c r="C96" s="1">
+      <c r="B96" s="6">
+        <v>5</v>
+      </c>
+      <c r="C96" s="7">
         <v>2020</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="6">
         <f>A96-DATE(YEAR(A96), 1, 0)</f>
         <v>150</v>
       </c>
-      <c r="E96" t="s">
-        <v>6</v>
-      </c>
-      <c r="F96" t="s">
+      <c r="E96" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F96" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I96" t="s">
+      <c r="G96" s="6"/>
+      <c r="H96" s="6"/>
+      <c r="I96" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="J96">
+      <c r="J96" s="6">
         <v>3</v>
       </c>
-      <c r="K96" t="s">
+      <c r="K96" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A97" s="2">
+      <c r="A97" s="8">
         <v>44026</v>
       </c>
-      <c r="B97">
+      <c r="B97" s="6">
         <v>7</v>
       </c>
-      <c r="C97" s="1">
+      <c r="C97" s="7">
         <v>2020</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="6">
         <f>A97-DATE(YEAR(A97), 1, 0)</f>
         <v>196</v>
       </c>
-      <c r="E97" t="s">
-        <v>6</v>
-      </c>
-      <c r="F97" t="s">
+      <c r="E97" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F97" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I97" t="s">
+      <c r="G97" s="6"/>
+      <c r="H97" s="6"/>
+      <c r="I97" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J97">
-        <v>1</v>
-      </c>
-      <c r="K97" t="s">
+      <c r="J97" s="6">
+        <v>1</v>
+      </c>
+      <c r="K97" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A98" s="2">
+      <c r="A98" s="8">
         <v>44028</v>
       </c>
-      <c r="B98">
+      <c r="B98" s="6">
         <v>7</v>
       </c>
-      <c r="C98" s="1">
+      <c r="C98" s="7">
         <v>2020</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="6">
         <f>A98-DATE(YEAR(A98), 1, 0)</f>
         <v>198</v>
       </c>
-      <c r="E98" t="s">
-        <v>6</v>
-      </c>
-      <c r="F98" t="s">
+      <c r="E98" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F98" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I98" t="s">
+      <c r="G98" s="6"/>
+      <c r="H98" s="6"/>
+      <c r="I98" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J98">
-        <v>1</v>
-      </c>
-      <c r="K98" t="s">
+      <c r="J98" s="6">
+        <v>1</v>
+      </c>
+      <c r="K98" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A99" s="2">
+      <c r="A99" s="8">
         <v>44037</v>
       </c>
-      <c r="B99">
+      <c r="B99" s="6">
         <v>7</v>
       </c>
-      <c r="C99" s="1">
+      <c r="C99" s="7">
         <v>2020</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="6">
         <f>A99-DATE(YEAR(A99), 1, 0)</f>
         <v>207</v>
       </c>
-      <c r="E99" t="s">
-        <v>6</v>
-      </c>
-      <c r="F99" t="s">
+      <c r="E99" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F99" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I99" t="s">
+      <c r="G99" s="6"/>
+      <c r="H99" s="6"/>
+      <c r="I99" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J99">
-        <v>1</v>
-      </c>
-      <c r="K99" t="s">
+      <c r="J99" s="6">
+        <v>1</v>
+      </c>
+      <c r="K99" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A100" s="2">
+      <c r="A100" s="8">
         <v>44038</v>
       </c>
-      <c r="B100">
+      <c r="B100" s="6">
         <v>7</v>
       </c>
-      <c r="C100" s="1">
+      <c r="C100" s="7">
         <v>2020</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="6">
         <f>A100-DATE(YEAR(A100), 1, 0)</f>
         <v>208</v>
       </c>
-      <c r="E100" t="s">
-        <v>6</v>
-      </c>
-      <c r="F100" t="s">
+      <c r="E100" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F100" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I100" t="s">
+      <c r="G100" s="6"/>
+      <c r="H100" s="6"/>
+      <c r="I100" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J100">
-        <v>1</v>
-      </c>
-      <c r="K100" t="s">
+      <c r="J100" s="6">
+        <v>1</v>
+      </c>
+      <c r="K100" s="6" t="s">
         <v>61</v>
       </c>
     </row>

</xml_diff>